<commit_message>
First snapshot of solarbank case
</commit_message>
<xml_diff>
--- a/BOM/BOM.xlsx
+++ b/BOM/BOM.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12300" activeTab="1"/>
+    <workbookView windowWidth="20490" windowHeight="7620" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="PCB_BOM" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="150">
   <si>
     <t>Reference,</t>
   </si>
@@ -472,6 +472,12 @@
   </si>
   <si>
     <t>https://sklep.msalamon.pl/produkt/panel-sloneczny-120x38mm-6v-100ma-06w/</t>
+  </si>
+  <si>
+    <t>Cell</t>
+  </si>
+  <si>
+    <t>https://botland.com.pl/akumulatory-li-pol-1s-37v/15643-akumulator-li-pol-akyga-3500mah-1s-37v-zlacze-jst-bec-gniazdo-68x55x6mm-5904422324438.html</t>
   </si>
 </sst>
 </file>
@@ -1101,7 +1107,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="26" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1111,14 +1117,11 @@
     <xf numFmtId="26" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="26" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="26" fontId="2" fillId="0" borderId="0" xfId="6">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="26" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="26" fontId="2" fillId="0" borderId="0" xfId="6">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="26" fontId="3" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment vertical="center"/>
@@ -1660,8 +1663,8 @@
   <sheetFormatPr defaultColWidth="10.2857142857143" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="41.1428571428571" customWidth="1"/>
-    <col min="2" max="2" width="6.85714285714286" style="3" customWidth="1"/>
-    <col min="3" max="3" width="24.4285714285714" style="3" customWidth="1"/>
+    <col min="2" max="2" width="6.85714285714286" style="1" customWidth="1"/>
+    <col min="3" max="3" width="24.4285714285714" style="1" customWidth="1"/>
     <col min="4" max="4" width="83.2857142857143" customWidth="1"/>
     <col min="5" max="5" width="255.714285714286" customWidth="1"/>
   </cols>
@@ -1687,16 +1690,16 @@
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="1">
         <v>9</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="3" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1704,16 +1707,16 @@
       <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="1">
         <v>8</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1721,16 +1724,16 @@
       <c r="A4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="1">
         <v>10</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D4" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1738,16 +1741,16 @@
       <c r="A5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="3">
-        <v>1</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="3" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1755,16 +1758,16 @@
       <c r="A6" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="3">
-        <v>1</v>
-      </c>
-      <c r="C6" s="3" t="s">
+      <c r="B6" s="1">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D6" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1772,16 +1775,16 @@
       <c r="A7" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="3">
-        <v>1</v>
-      </c>
-      <c r="C7" s="3" t="s">
+      <c r="B7" s="1">
+        <v>1</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D7" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="5" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1789,16 +1792,16 @@
       <c r="A8" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="1">
         <v>2</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="1" t="s">
         <v>25</v>
       </c>
       <c r="D8" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="3" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1806,16 +1809,16 @@
       <c r="A9" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="1">
         <v>2</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D9" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="3" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1823,10 +1826,10 @@
       <c r="A10" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="1">
         <v>2</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="1" t="s">
         <v>33</v>
       </c>
       <c r="D10" t="s">
@@ -1840,10 +1843,10 @@
       <c r="A11" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="3">
-        <v>1</v>
-      </c>
-      <c r="C11" s="3" t="s">
+      <c r="B11" s="1">
+        <v>1</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D11" t="s">
@@ -1857,10 +1860,10 @@
       <c r="A12" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="3">
-        <v>1</v>
-      </c>
-      <c r="C12" s="3" t="s">
+      <c r="B12" s="1">
+        <v>1</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>41</v>
       </c>
       <c r="D12" t="s">
@@ -1874,10 +1877,10 @@
       <c r="A13" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="1">
         <v>2</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="1" t="s">
         <v>45</v>
       </c>
       <c r="D13" t="s">
@@ -1891,10 +1894,10 @@
       <c r="A14" t="s">
         <v>48</v>
       </c>
-      <c r="B14" s="3">
-        <v>1</v>
-      </c>
-      <c r="C14" s="3" t="s">
+      <c r="B14" s="1">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>49</v>
       </c>
       <c r="D14" t="s">
@@ -1908,16 +1911,16 @@
       <c r="A15" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="1">
         <v>4</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="1" t="s">
         <v>53</v>
       </c>
       <c r="D15" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1925,10 +1928,10 @@
       <c r="A16" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="3">
-        <v>1</v>
-      </c>
-      <c r="C16" s="3" t="s">
+      <c r="B16" s="1">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>57</v>
       </c>
       <c r="D16" t="s">
@@ -1942,16 +1945,16 @@
       <c r="A17" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="3">
-        <v>1</v>
-      </c>
-      <c r="C17" s="3" t="s">
+      <c r="B17" s="1">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>61</v>
       </c>
       <c r="D17" t="s">
         <v>54</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="3" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1959,10 +1962,10 @@
       <c r="A18" t="s">
         <v>63</v>
       </c>
-      <c r="B18" s="3">
+      <c r="B18" s="1">
         <v>3</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="1" t="s">
         <v>64</v>
       </c>
       <c r="D18" t="s">
@@ -1976,10 +1979,10 @@
       <c r="A19" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="3">
-        <v>1</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="B19" s="1">
+        <v>1</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>68</v>
       </c>
       <c r="D19" t="s">
@@ -1993,10 +1996,10 @@
       <c r="A20" t="s">
         <v>70</v>
       </c>
-      <c r="B20" s="3">
-        <v>1</v>
-      </c>
-      <c r="C20" s="3" t="s">
+      <c r="B20" s="1">
+        <v>1</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>71</v>
       </c>
       <c r="D20" t="s">
@@ -2010,10 +2013,10 @@
       <c r="A21" t="s">
         <v>73</v>
       </c>
-      <c r="B21" s="3">
+      <c r="B21" s="1">
         <v>8</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="1" t="s">
         <v>74</v>
       </c>
       <c r="D21" t="s">
@@ -2027,10 +2030,10 @@
       <c r="A22" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="3">
-        <v>1</v>
-      </c>
-      <c r="C22" s="3" t="s">
+      <c r="B22" s="1">
+        <v>1</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>77</v>
       </c>
       <c r="D22" t="s">
@@ -2044,10 +2047,10 @@
       <c r="A23" t="s">
         <v>79</v>
       </c>
-      <c r="B23" s="3">
-        <v>1</v>
-      </c>
-      <c r="C23" s="3" t="s">
+      <c r="B23" s="1">
+        <v>1</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>80</v>
       </c>
       <c r="D23" t="s">
@@ -2061,10 +2064,10 @@
       <c r="A24" t="s">
         <v>82</v>
       </c>
-      <c r="B24" s="3">
+      <c r="B24" s="1">
         <v>3</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="1" t="s">
         <v>83</v>
       </c>
       <c r="D24" t="s">
@@ -2078,10 +2081,10 @@
       <c r="A25" t="s">
         <v>85</v>
       </c>
-      <c r="B25" s="3">
-        <v>1</v>
-      </c>
-      <c r="C25" s="3" t="s">
+      <c r="B25" s="1">
+        <v>1</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>86</v>
       </c>
       <c r="D25" t="s">
@@ -2095,10 +2098,10 @@
       <c r="A26" t="s">
         <v>88</v>
       </c>
-      <c r="B26" s="3">
-        <v>1</v>
-      </c>
-      <c r="C26" s="3" t="s">
+      <c r="B26" s="1">
+        <v>1</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>89</v>
       </c>
       <c r="D26" t="s">
@@ -2112,10 +2115,10 @@
       <c r="A27" t="s">
         <v>91</v>
       </c>
-      <c r="B27" s="3">
-        <v>1</v>
-      </c>
-      <c r="C27" s="3" t="s">
+      <c r="B27" s="1">
+        <v>1</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>92</v>
       </c>
       <c r="D27" t="s">
@@ -2129,10 +2132,10 @@
       <c r="A28" t="s">
         <v>94</v>
       </c>
-      <c r="B28" s="3">
-        <v>1</v>
-      </c>
-      <c r="C28" s="3">
+      <c r="B28" s="1">
+        <v>1</v>
+      </c>
+      <c r="C28" s="1">
         <v>100</v>
       </c>
       <c r="D28" t="s">
@@ -2146,10 +2149,10 @@
       <c r="A29" t="s">
         <v>96</v>
       </c>
-      <c r="B29" s="3">
+      <c r="B29" s="1">
         <v>2</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="1" t="s">
         <v>97</v>
       </c>
       <c r="D29" t="s">
@@ -2163,10 +2166,10 @@
       <c r="A30" t="s">
         <v>99</v>
       </c>
-      <c r="B30" s="3">
-        <v>1</v>
-      </c>
-      <c r="C30" s="3" t="s">
+      <c r="B30" s="1">
+        <v>1</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>100</v>
       </c>
       <c r="D30" t="s">
@@ -2180,10 +2183,10 @@
       <c r="A31" t="s">
         <v>102</v>
       </c>
-      <c r="B31" s="3">
-        <v>1</v>
-      </c>
-      <c r="C31" s="3" t="s">
+      <c r="B31" s="1">
+        <v>1</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>103</v>
       </c>
       <c r="D31" t="s">
@@ -2197,10 +2200,10 @@
       <c r="A32" t="s">
         <v>105</v>
       </c>
-      <c r="B32" s="3">
-        <v>1</v>
-      </c>
-      <c r="C32" s="3" t="s">
+      <c r="B32" s="1">
+        <v>1</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>106</v>
       </c>
       <c r="D32" t="s">
@@ -2211,10 +2214,10 @@
       <c r="A33" t="s">
         <v>107</v>
       </c>
-      <c r="B33" s="3">
+      <c r="B33" s="1">
         <v>3</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="1" t="s">
         <v>108</v>
       </c>
       <c r="D33" t="s">
@@ -2228,10 +2231,10 @@
       <c r="A34" t="s">
         <v>110</v>
       </c>
-      <c r="B34" s="3">
-        <v>1</v>
-      </c>
-      <c r="C34" s="3" t="s">
+      <c r="B34" s="1">
+        <v>1</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>111</v>
       </c>
       <c r="D34" t="s">
@@ -2245,10 +2248,10 @@
       <c r="A35" t="s">
         <v>113</v>
       </c>
-      <c r="B35" s="3">
-        <v>1</v>
-      </c>
-      <c r="C35" s="3" t="s">
+      <c r="B35" s="1">
+        <v>1</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>114</v>
       </c>
       <c r="D35" t="s">
@@ -2262,16 +2265,16 @@
       <c r="A36" t="s">
         <v>117</v>
       </c>
-      <c r="B36" s="3">
-        <v>1</v>
-      </c>
-      <c r="C36" s="3" t="s">
+      <c r="B36" s="1">
+        <v>1</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>118</v>
       </c>
       <c r="D36" t="s">
         <v>119</v>
       </c>
-      <c r="E36" s="5" t="s">
+      <c r="E36" s="3" t="s">
         <v>120</v>
       </c>
     </row>
@@ -2279,16 +2282,16 @@
       <c r="A37" t="s">
         <v>121</v>
       </c>
-      <c r="B37" s="3">
-        <v>1</v>
-      </c>
-      <c r="C37" s="3" t="s">
+      <c r="B37" s="1">
+        <v>1</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>122</v>
       </c>
       <c r="D37" t="s">
         <v>123</v>
       </c>
-      <c r="E37" s="5" t="s">
+      <c r="E37" s="3" t="s">
         <v>59</v>
       </c>
     </row>
@@ -2296,10 +2299,10 @@
       <c r="A38" t="s">
         <v>124</v>
       </c>
-      <c r="B38" s="3">
-        <v>1</v>
-      </c>
-      <c r="C38" s="3" t="s">
+      <c r="B38" s="1">
+        <v>1</v>
+      </c>
+      <c r="C38" s="1" t="s">
         <v>125</v>
       </c>
       <c r="D38" t="s">
@@ -2313,10 +2316,10 @@
       <c r="A39" t="s">
         <v>128</v>
       </c>
-      <c r="B39" s="3">
-        <v>1</v>
-      </c>
-      <c r="C39" s="3" t="s">
+      <c r="B39" s="1">
+        <v>1</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>129</v>
       </c>
       <c r="D39" t="s">
@@ -2330,10 +2333,10 @@
       <c r="A40" t="s">
         <v>132</v>
       </c>
-      <c r="B40" s="3">
-        <v>1</v>
-      </c>
-      <c r="C40" s="3" t="s">
+      <c r="B40" s="1">
+        <v>1</v>
+      </c>
+      <c r="C40" s="1" t="s">
         <v>133</v>
       </c>
       <c r="D40" t="s">
@@ -2363,7 +2366,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="14.2857142857143" customWidth="1"/>
@@ -2438,11 +2441,25 @@
       <c r="B9" s="1">
         <v>2</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="3" t="s">
         <v>147</v>
       </c>
     </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>148</v>
+      </c>
+      <c r="B11" s="1">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>149</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C9" r:id="rId1" display="https://sklep.msalamon.pl/produkt/panel-sloneczny-120x38mm-6v-100ma-06w/"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
SolarBank housing is almost ready
Need to add heat-set threads holes
</commit_message>
<xml_diff>
--- a/BOM/BOM.xlsx
+++ b/BOM/BOM.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620" activeTab="1"/>
+    <workbookView windowWidth="27945" windowHeight="12300" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="PCB_BOM" sheetId="1" r:id="rId1"/>
@@ -509,7 +509,7 @@
     <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -517,7 +517,7 @@
     <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -977,10 +977,10 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="26" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="26" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="26" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="26" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
@@ -1117,13 +1117,13 @@
     <xf numFmtId="26" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="26" fontId="2" fillId="0" borderId="0" xfId="6">
+    <xf numFmtId="26" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="26" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="26" fontId="3" fillId="0" borderId="0" xfId="6" applyFont="1">
+    <xf numFmtId="26" fontId="3" fillId="0" borderId="0" xfId="6">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1699,7 +1699,7 @@
       <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="5" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1716,7 +1716,7 @@
       <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="5" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
       <c r="D4" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="3" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1750,7 +1750,7 @@
       <c r="D5" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="5" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1767,7 +1767,7 @@
       <c r="D6" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="3" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
       <c r="D7" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="3" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
       <c r="D8" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="5" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1818,7 +1818,7 @@
       <c r="D9" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="5" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       <c r="D15" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="5" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       <c r="D17" t="s">
         <v>54</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
       <c r="D36" t="s">
         <v>119</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" s="5" t="s">
         <v>120</v>
       </c>
     </row>
@@ -2291,7 +2291,7 @@
       <c r="D37" t="s">
         <v>123</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" s="5" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>

<commit_message>
finishing touches to the housing
</commit_message>
<xml_diff>
--- a/BOM/BOM.xlsx
+++ b/BOM/BOM.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="152">
   <si>
     <t>Reference,</t>
   </si>
@@ -123,7 +123,7 @@
     <t>Diode_SMD:D_SMA</t>
   </si>
   <si>
-    <t>https://www.tme.eu/pl/details/ss32bf-dc/diody-schottky-smd/dc-components/ss32bf/</t>
+    <t>https://www.tme.eu/pl/details/b340a-13-f/diody-schottky-smd/diodes-incorporated</t>
   </si>
   <si>
     <t>IC1,IC2,</t>
@@ -135,7 +135,7 @@
     <t>KiCad:TPS630701RNMR</t>
   </si>
   <si>
-    <t>https://www.mouser.pl/pl/ProductDetail/Texas-Instruments/TPS630701RNMR?qs=LuYMPh7GGMTyE4ON9PhzXw%3D%3D&amp;utm_id=22436684815&amp;utm_source=google&amp;utm_medium=cpc&amp;utm_marketing_tactic=emeacorp&amp;gad_source=1&amp;gad_campaignid=22426729329&amp;gbraid=0AAAAADn_wf3XMHQ6zRhB7voaiurS8BXmv&amp;gclid=CjwKCAjwn67VBhBnEiwAXUIN1THLO1qN-YgxaSPJNR99Heb35tPZ9mEgLFExLuTE6wJ6alpddn_etxoCz_UQAvD_BwE</t>
+    <t>https://www.digikey.pl/en/products/detail/texas-instruments/TPS63070RNMR/6217416</t>
   </si>
   <si>
     <t>J1,</t>
@@ -183,9 +183,6 @@
     <t>Inductor_SMD:L_Coilcraft_XAL5030-XXX</t>
   </si>
   <si>
-    <t>https://www.coilcraft.com/en-us/products/power/shielded-inductors/molded-inductor/xfl/xfl4020/xfl4020-102/</t>
-  </si>
-  <si>
     <t>Q1,Q3,Q4,Q5,</t>
   </si>
   <si>
@@ -195,7 +192,7 @@
     <t>Package_TO_SOT_SMD:SOT-23</t>
   </si>
   <si>
-    <t>https://www.tme.eu/pl/katalog/?queryPhrase=DMP3099L</t>
+    <t>https://www.tme.eu/pl/details/2n7002-dio/tranzystory-z-kanalem-n-smd/diotec-semiconductor/2n7002</t>
   </si>
   <si>
     <t>Q2,</t>
@@ -478,6 +475,15 @@
   </si>
   <si>
     <t>https://botland.com.pl/akumulatory-li-pol-1s-37v/15643-akumulator-li-pol-akyga-3500mah-1s-37v-zlacze-jst-bec-gniazdo-68x55x6mm-5904422324438.html</t>
+  </si>
+  <si>
+    <t>M2 heatset inserts &amp; bolts</t>
+  </si>
+  <si>
+    <t>https://www.ruthex.de/en/products/ruthex-gewindeeinsatz-m2-70-stuck-rx-m2x4-messing-gewindebuchsen?srsltid=AU7gw4X9_ky8HLKVFD2MPkiC0q8hMxmiFJ4ZEjWMObGkNThVd5x1F2D8</t>
+  </si>
+  <si>
+    <t>https://rc-team.pl/wszystkie-czesci-maverick/144486-maverick-sruby-m2x15mm-countersunk-screw-5700135347456-534745.html</t>
   </si>
 </sst>
 </file>
@@ -1107,7 +1113,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="26" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1120,11 +1126,17 @@
     <xf numFmtId="26" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="26" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="26" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="26" fontId="3" fillId="0" borderId="0" xfId="6">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="26" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="26" fontId="3" fillId="0" borderId="0" xfId="6">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1682,7 +1694,7 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1699,7 +1711,7 @@
       <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1716,7 +1728,7 @@
       <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1750,7 +1762,7 @@
       <c r="D5" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1801,7 +1813,7 @@
       <c r="D8" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1818,7 +1830,7 @@
       <c r="D9" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1835,7 +1847,7 @@
       <c r="D10" t="s">
         <v>34</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="6" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1903,234 +1915,234 @@
       <c r="D14" t="s">
         <v>50</v>
       </c>
-      <c r="E14" t="s">
-        <v>51</v>
+      <c r="E14" s="6" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B15" s="1">
         <v>4</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" t="s">
         <v>53</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" s="6" t="s">
         <v>54</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="1">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="1">
-        <v>1</v>
-      </c>
-      <c r="C16" s="1" t="s">
+      <c r="D16" t="s">
         <v>57</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>58</v>
-      </c>
-      <c r="E16" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="1">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="1">
-        <v>1</v>
-      </c>
-      <c r="C17" s="1" t="s">
+      <c r="D17" t="s">
+        <v>53</v>
+      </c>
+      <c r="E17" s="6" t="s">
         <v>61</v>
-      </c>
-      <c r="D17" t="s">
-        <v>54</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B18" s="1">
         <v>3</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" t="s">
         <v>64</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>65</v>
-      </c>
-      <c r="E18" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" s="1">
+        <v>1</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="1">
-        <v>1</v>
-      </c>
-      <c r="C19" s="1" t="s">
+      <c r="D19" t="s">
+        <v>64</v>
+      </c>
+      <c r="E19" t="s">
         <v>68</v>
-      </c>
-      <c r="D19" t="s">
-        <v>65</v>
-      </c>
-      <c r="E19" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="1">
+        <v>1</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B20" s="1">
-        <v>1</v>
-      </c>
-      <c r="C20" s="1" t="s">
+      <c r="D20" t="s">
+        <v>64</v>
+      </c>
+      <c r="E20" t="s">
         <v>71</v>
-      </c>
-      <c r="D20" t="s">
-        <v>65</v>
-      </c>
-      <c r="E20" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B21" s="1">
         <v>8</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D21" t="s">
+        <v>64</v>
+      </c>
+      <c r="E21" t="s">
         <v>74</v>
-      </c>
-      <c r="D21" t="s">
-        <v>65</v>
-      </c>
-      <c r="E21" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
+        <v>75</v>
+      </c>
+      <c r="B22" s="1">
+        <v>1</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="1">
-        <v>1</v>
-      </c>
-      <c r="C22" s="1" t="s">
+      <c r="D22" t="s">
+        <v>64</v>
+      </c>
+      <c r="E22" t="s">
         <v>77</v>
-      </c>
-      <c r="D22" t="s">
-        <v>65</v>
-      </c>
-      <c r="E22" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
+        <v>78</v>
+      </c>
+      <c r="B23" s="1">
+        <v>1</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B23" s="1">
-        <v>1</v>
-      </c>
-      <c r="C23" s="1" t="s">
+      <c r="D23" t="s">
+        <v>64</v>
+      </c>
+      <c r="E23" t="s">
         <v>80</v>
-      </c>
-      <c r="D23" t="s">
-        <v>65</v>
-      </c>
-      <c r="E23" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B24" s="1">
         <v>3</v>
       </c>
       <c r="C24" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D24" t="s">
+        <v>64</v>
+      </c>
+      <c r="E24" t="s">
         <v>83</v>
-      </c>
-      <c r="D24" t="s">
-        <v>65</v>
-      </c>
-      <c r="E24" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
+        <v>84</v>
+      </c>
+      <c r="B25" s="1">
+        <v>1</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B25" s="1">
-        <v>1</v>
-      </c>
-      <c r="C25" s="1" t="s">
+      <c r="D25" t="s">
+        <v>64</v>
+      </c>
+      <c r="E25" t="s">
         <v>86</v>
-      </c>
-      <c r="D25" t="s">
-        <v>65</v>
-      </c>
-      <c r="E25" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
+        <v>87</v>
+      </c>
+      <c r="B26" s="1">
+        <v>1</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B26" s="1">
-        <v>1</v>
-      </c>
-      <c r="C26" s="1" t="s">
+      <c r="D26" t="s">
+        <v>64</v>
+      </c>
+      <c r="E26" t="s">
         <v>89</v>
-      </c>
-      <c r="D26" t="s">
-        <v>65</v>
-      </c>
-      <c r="E26" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
+        <v>90</v>
+      </c>
+      <c r="B27" s="1">
+        <v>1</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B27" s="1">
-        <v>1</v>
-      </c>
-      <c r="C27" s="1" t="s">
+      <c r="D27" t="s">
+        <v>64</v>
+      </c>
+      <c r="E27" t="s">
         <v>92</v>
-      </c>
-      <c r="D27" t="s">
-        <v>65</v>
-      </c>
-      <c r="E27" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B28" s="1">
         <v>1</v>
@@ -2139,211 +2151,211 @@
         <v>100</v>
       </c>
       <c r="D28" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E28" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B29" s="1">
         <v>2</v>
       </c>
       <c r="C29" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D29" t="s">
+        <v>64</v>
+      </c>
+      <c r="E29" t="s">
         <v>97</v>
-      </c>
-      <c r="D29" t="s">
-        <v>65</v>
-      </c>
-      <c r="E29" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
+        <v>98</v>
+      </c>
+      <c r="B30" s="1">
+        <v>1</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B30" s="1">
-        <v>1</v>
-      </c>
-      <c r="C30" s="1" t="s">
+      <c r="D30" t="s">
+        <v>64</v>
+      </c>
+      <c r="E30" t="s">
         <v>100</v>
-      </c>
-      <c r="D30" t="s">
-        <v>65</v>
-      </c>
-      <c r="E30" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
+        <v>101</v>
+      </c>
+      <c r="B31" s="1">
+        <v>1</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B31" s="1">
-        <v>1</v>
-      </c>
-      <c r="C31" s="1" t="s">
+      <c r="D31" t="s">
+        <v>64</v>
+      </c>
+      <c r="E31" t="s">
         <v>103</v>
-      </c>
-      <c r="D31" t="s">
-        <v>65</v>
-      </c>
-      <c r="E31" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
+        <v>104</v>
+      </c>
+      <c r="B32" s="1">
+        <v>1</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B32" s="1">
-        <v>1</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>106</v>
-      </c>
       <c r="D32" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B33" s="1">
         <v>3</v>
       </c>
       <c r="C33" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D33" t="s">
+        <v>64</v>
+      </c>
+      <c r="E33" t="s">
         <v>108</v>
-      </c>
-      <c r="D33" t="s">
-        <v>65</v>
-      </c>
-      <c r="E33" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
+        <v>109</v>
+      </c>
+      <c r="B34" s="1">
+        <v>1</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B34" s="1">
-        <v>1</v>
-      </c>
-      <c r="C34" s="1" t="s">
+      <c r="D34" t="s">
+        <v>64</v>
+      </c>
+      <c r="E34" t="s">
         <v>111</v>
-      </c>
-      <c r="D34" t="s">
-        <v>65</v>
-      </c>
-      <c r="E34" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
+        <v>112</v>
+      </c>
+      <c r="B35" s="1">
+        <v>1</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B35" s="1">
-        <v>1</v>
-      </c>
-      <c r="C35" s="1" t="s">
+      <c r="D35" t="s">
         <v>114</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>115</v>
-      </c>
-      <c r="E35" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
+        <v>116</v>
+      </c>
+      <c r="B36" s="1">
+        <v>1</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B36" s="1">
-        <v>1</v>
-      </c>
-      <c r="C36" s="1" t="s">
+      <c r="D36" t="s">
         <v>118</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
+        <v>120</v>
+      </c>
+      <c r="B37" s="1">
+        <v>1</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B37" s="1">
-        <v>1</v>
-      </c>
-      <c r="C37" s="1" t="s">
+      <c r="D37" t="s">
         <v>122</v>
       </c>
-      <c r="D37" t="s">
-        <v>123</v>
-      </c>
-      <c r="E37" s="5" t="s">
-        <v>59</v>
+      <c r="E37" s="6" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
+        <v>123</v>
+      </c>
+      <c r="B38" s="1">
+        <v>1</v>
+      </c>
+      <c r="C38" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="B38" s="1">
-        <v>1</v>
-      </c>
-      <c r="C38" s="1" t="s">
+      <c r="D38" t="s">
         <v>125</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>126</v>
-      </c>
-      <c r="E38" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
+        <v>127</v>
+      </c>
+      <c r="B39" s="1">
+        <v>1</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B39" s="1">
-        <v>1</v>
-      </c>
-      <c r="C39" s="1" t="s">
+      <c r="D39" t="s">
         <v>129</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>130</v>
-      </c>
-      <c r="E39" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
+        <v>131</v>
+      </c>
+      <c r="B40" s="1">
+        <v>1</v>
+      </c>
+      <c r="C40" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B40" s="1">
-        <v>1</v>
-      </c>
-      <c r="C40" s="1" t="s">
+      <c r="D40" t="s">
         <v>133</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>134</v>
-      </c>
-      <c r="E40" t="s">
-        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -2352,11 +2364,13 @@
     <hyperlink ref="E3" r:id="rId2" display="https://www.tme.eu/pl/details/grm31cr61e226ke15l/kondensatory-mlcc-smd/murata/"/>
     <hyperlink ref="E4" r:id="rId3" display="https://www.tme.eu/pl/details/cl31a106kahnnne/kondensatory-mlcc-smd/samsung/"/>
     <hyperlink ref="E5" r:id="rId4" display="https://www.tme.eu/pl/details/cl31a475kahnnne/kondensatory-mlcc-smd/samsung/"/>
-    <hyperlink ref="E9" r:id="rId5" display="https://www.tme.eu/pl/details/ss32bf-dc/diody-schottky-smd/dc-components/ss32bf/"/>
+    <hyperlink ref="E9" r:id="rId5" display="https://www.tme.eu/pl/details/b340a-13-f/diody-schottky-smd/diodes-incorporated" tooltip="https://www.tme.eu/pl/details/b340a-13-f/diody-schottky-smd/diodes-incorporated"/>
     <hyperlink ref="E8" r:id="rId6" display="https://www.tme.eu/pl/details/of-smd3216r/diody-led-smd-kolorowe/optoflash/"/>
     <hyperlink ref="E17" r:id="rId7" display="https://www.tme.eu/pl/details/dmp3099l-7/tranzystory-z-kanalem-p-smd/diodes-incorporated/"/>
-    <hyperlink ref="E15" r:id="rId8" display="https://www.tme.eu/pl/katalog/?queryPhrase=DMP3099L"/>
+    <hyperlink ref="E15" r:id="rId8" display="https://www.tme.eu/pl/details/2n7002-dio/tranzystory-z-kanalem-n-smd/diotec-semiconductor/2n7002" tooltip="https://www.tme.eu/pl/details/2n7002-dio/tranzystory-z-kanalem-n-smd/diotec-semiconductor/2n7002"/>
     <hyperlink ref="E36" r:id="rId9" display="https://www.mouser.pl/pl/ProductDetail/Microchip-Technology/MCP4018T-103E-LTY?qs=savM97goi5hGuILh2wIQ1w%3D%3D"/>
+    <hyperlink ref="E14" r:id="rId10" display="https://www.digikey.pl/en/products/detail/texas-instruments/TPS63070RNMR/6217416"/>
+    <hyperlink ref="E10" r:id="rId10" display="https://www.digikey.pl/en/products/detail/texas-instruments/TPS63070RNMR/6217416"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -2366,7 +2380,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="14.2857142857143" customWidth="1"/>
@@ -2376,7 +2390,7 @@
   <sheetData>
     <row r="1" ht="26.25" spans="1:3">
       <c r="A1" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -2387,78 +2401,101 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
         <v>138</v>
-      </c>
-      <c r="B3" s="1">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
         <v>140</v>
-      </c>
-      <c r="B4" s="1">
-        <v>1</v>
-      </c>
-      <c r="C4" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
+        <v>141</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
         <v>142</v>
-      </c>
-      <c r="B5" s="1">
-        <v>1</v>
-      </c>
-      <c r="C5" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B7" s="1">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
         <v>144</v>
-      </c>
-      <c r="B7" s="1">
-        <v>1</v>
-      </c>
-      <c r="C7" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B9" s="1">
         <v>2</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
+        <v>147</v>
+      </c>
+      <c r="B11" s="1">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
         <v>148</v>
       </c>
-      <c r="B11" s="1">
-        <v>1</v>
-      </c>
-      <c r="C11" t="s">
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="4" t="s">
         <v>149</v>
       </c>
+      <c r="B13" s="5">
+        <v>4</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="4"/>
+      <c r="B14" s="5"/>
+      <c r="C14" t="s">
+        <v>151</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="C9" r:id="rId1" display="https://sklep.msalamon.pl/produkt/panel-sloneczny-120x38mm-6v-100ma-06w/"/>
+    <hyperlink ref="C13" r:id="rId2" display="https://www.ruthex.de/en/products/ruthex-gewindeeinsatz-m2-70-stuck-rx-m2x4-messing-gewindebuchsen?srsltid=AU7gw4X9_ky8HLKVFD2MPkiC0q8hMxmiFJ4ZEjWMObGkNThVd5x1F2D8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>